<commit_message>
(v3.0.1.9106) Fix trade names of combinations filed under a single agent, and remove non-synonyms from `antimicrobials` (#315)
</commit_message>
<xml_diff>
--- a/data-raw/datasets/antimicrobials.xlsx
+++ b/data-raw/datasets/antimicrobials.xlsx
@@ -483,7 +483,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>aminacyl,aminopar,aminosalyl,aminox,apacil,deapasil,entepas,gabbropas,granupas,helipidyl,hellipidyl,nemasol,nippas,osacyl,pamacyl,pamisyl,paramisan,paramycin,parasal,parasalicil,parasalindon,pasade,pasalon,pasara,pascorbic,pasdium,pasem,paser,pasmed,pasnal,pasnodia,pasolac,passodico,pharmakon,propasa,rezipas,salvis,sanipirol,sanipriol,sodiopas,spectrum</t>
+          <t>aminacyl,aminopar,aminosalyl,aminox,apacil,deapasil,entepas,gabbropas,granupas,helipidyl,hellipidyl,nemasol,nippas,osacyl,pamacyl,pamisyl,paramisan,paramycin,parasal,parasalicil,parasalindon,pasade,pasalon,pasara,pascorbic,pasdium,pasem,paser,pasmed,pasnal,pasnodia,pasolac,passodico,propasa,rezipas,salvis,sanipirol,sanipriol,sodiopas</t>
         </is>
       </c>
       <c r="J2">
@@ -727,7 +727,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>amikacillin,amikacina,amikacine,amikacinum,amikavet,amikin,amikozit,amukin,arikace,briclin,butirosins,kaminax,lukadin,mikavir,potentox,prestwick</t>
+          <t>amikacillin,amikacina,amikacine,amikacinum,amikavet,amikin,amikozit,amukin,arikace,briclin,butirosins,kaminax,lukadin,mikavir,potentox</t>
         </is>
       </c>
       <c r="J6" t="e">
@@ -3107,7 +3107,7 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>blenamax,blenoxane,bleocin,bleomicin,bleomicina,bleomycine,bleomycins,bleomycinum,blexane,nbleomycinamide</t>
+          <t>blenamax,blenoxane,bleocin,bleomicin,bleomicina,bleomycine,bleomycins,bleomycinum,blexane</t>
         </is>
       </c>
       <c r="J45" t="e">
@@ -3791,7 +3791,7 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>alenfral,alfacet,alfatil,ceclor,cefachlor,cefaclorum,cefeaclor,cephaclor,compound,distaclor,keflor,kefolor,kefral,keftab,keftid,lilly,lopac,panacef,panoral,raniclor</t>
+          <t>alenfral,alfacet,alfatil,ceclor,cefachlor,cefaclorum,cefeaclor,cephaclor,compound,distaclor,keflor,kefolor,kefral,keftab,keftid,lilly,panacef,panoral,raniclor</t>
         </is>
       </c>
       <c r="J56">
@@ -4975,7 +4975,7 @@
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>exblifep</t>
         </is>
       </c>
       <c r="J75" t="e">
@@ -14041,7 +14041,7 @@
       </c>
       <c r="I222" t="inlineStr">
         <is>
-          <t>amudane,delmofulvina,epigriseofulvin,fulcin,fulcine,fulvicin,fulvidex,fulvina,fulvinil,fulvistatin,fungivin,greosin,gresfeed,gricin,grifulin,grifulvin,grisactin,griscofulvin,grisefuline,griseo,griseofulviin,griseofulvina,griseofulvine,griseofulvinum,griseomix,griseostatin,grisetin,grisofulvin,grisovin,grisowen,grizeofulvin,grysio,guservin,lamoryl,likuden,likunden,murfulvin,poncyl,spiro,spirofulvin,xuanjing</t>
+          <t>amudane,delmofulvina,epigriseofulvin,fulcin,fulcine,fulvicin,fulvidex,fulvina,fulvinil,fulvistatin,fungivin,greosin,gresfeed,gricin,grifulin,grifulvin,grisactin,griscofulvin,grisefuline,griseo,griseofulviin,griseofulvina,griseofulvine,griseofulvinum,griseomix,griseostatin,grisetin,grisofulvin,grisovin,grisowen,grizeofulvin,grysio,guservin,lamoryl,likuden,likunden,murfulvin,poncyl,spirofulvin,xuanjing</t>
         </is>
       </c>
       <c r="J222">
@@ -14463,7 +14463,7 @@
       </c>
       <c r="I229" t="inlineStr">
         <is>
-          <t>imipemide,imipenemum,imipenen,primaxin,recarbrio,tienam,tienamycin</t>
+          <t>imipemide,imipenemum,imipenen,primaxin,tienam,tienamycin</t>
         </is>
       </c>
       <c r="J229" t="e">
@@ -14581,7 +14581,7 @@
       </c>
       <c r="I231" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>recarbrio</t>
         </is>
       </c>
       <c r="J231" t="e">
@@ -15331,7 +15331,7 @@
       </c>
       <c r="I243" t="inlineStr">
         <is>
-          <t>brizoral,ethanone,extina,fungarest,fungoral,ketaconazole,ketocanazole,ketoconazol,ketoconazolum,ketodan,ketoderm,ketoisdin,ketozole,kuric,levoketoconazole,nizoral,normocort,panfungol,piperazine,recorlev,sebazole,teryzolin,terzolin,tocris,xolegel</t>
+          <t>brizoral,ethanone,extina,fungarest,fungoral,ketaconazole,ketocanazole,ketoconazol,ketoconazolum,ketodan,ketoderm,ketoisdin,ketozole,kuric,levoketoconazole,nizoral,normocort,panfungol,piperazine,recorlev,sebazole,teryzolin,terzolin,xolegel</t>
         </is>
       </c>
       <c r="J243">
@@ -21653,7 +21653,7 @@
       </c>
       <c r="I346" t="inlineStr">
         <is>
-          <t>penmalin,pentcillin,peperacillin,peracin,piperacilina,piperacillina,piperacilline,piperacillinhydrate,piperacillinum,pipercillin,pipracil,tazocin</t>
+          <t>penmalin,pentcillin,peperacillin,peracin,piperacilina,piperacillina,piperacilline,piperacillinhydrate,piperacillinum,pipercillin,pipracil</t>
         </is>
       </c>
       <c r="J346" t="e">
@@ -21777,7 +21777,7 @@
       </c>
       <c r="I348" t="inlineStr">
         <is>
-          <t>piptazobactam,tazonam,zobactin,zosyn</t>
+          <t>piptazobactam,tazocin,tazonam,zobactin,zosyn</t>
         </is>
       </c>
       <c r="J348" t="e">
@@ -28163,7 +28163,7 @@
       </c>
       <c r="I451" t="inlineStr">
         <is>
-          <t>exblifep,tazobactamsalt,tazobactamum,tazobactum</t>
+          <t>tazobactamsalt,tazobactamum,tazobactum</t>
         </is>
       </c>
       <c r="J451" t="e">
@@ -29397,7 +29397,7 @@
       </c>
       <c r="I471" t="inlineStr">
         <is>
-          <t>alaninamide,bryamycin,gargon,pharmakon,prestwick,sporangiomycin,thiactin,tiostrepton</t>
+          <t>alaninamide,bryamycin,gargon,sporangiomycin,thiactin,tiostrepton</t>
         </is>
       </c>
       <c r="J471" t="e">
@@ -29517,7 +29517,7 @@
       </c>
       <c r="I473" t="inlineStr">
         <is>
-          <t>ticar,ticarcilina,ticarcilline,ticarcillinum,timentin</t>
+          <t>ticar,ticarcilina,ticarcilline,ticarcillinum</t>
         </is>
       </c>
       <c r="J473" t="e">
@@ -29581,7 +29581,7 @@
       </c>
       <c r="I474" t="inlineStr">
         <is>
-          <t>augpenin</t>
+          <t>augpenin,timentin</t>
         </is>
       </c>
       <c r="J474" t="e">
@@ -31455,7 +31455,7 @@
       </c>
       <c r="I505" t="inlineStr">
         <is>
-          <t>nuzolvence,spiro,zoliflodacina,zoliflodacine</t>
+          <t>nuzolvence,zoliflodacina,zoliflodacine</t>
         </is>
       </c>
       <c r="J505" t="e">
@@ -31513,7 +31513,7 @@
       </c>
       <c r="I506" t="inlineStr">
         <is>
-          <t>bleomycetin,boanmycin,nbleomycinamide,pingyangmycin</t>
+          <t>bleomycetin,boanmycin,pingyangmycin</t>
         </is>
       </c>
       <c r="J506" t="e">

</xml_diff>